<commit_message>
Save in between version as this one rendeerd
</commit_message>
<xml_diff>
--- a/data/derived/Combined_data.xlsx
+++ b/data/derived/Combined_data.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:IH121"/>
+  <dimension ref="A1:II121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="11" max="11" width="20.7109375" style="2" customWidth="1"/>
@@ -1552,25 +1552,30 @@
       </c>
       <c r="ID1" s="1" t="inlineStr">
         <is>
+          <t>Site_type_detail</t>
+        </is>
+      </c>
+      <c r="IE1" s="1" t="inlineStr">
+        <is>
           <t>Substrate_index_after</t>
         </is>
       </c>
-      <c r="IE1" s="1" t="inlineStr">
+      <c r="IF1" s="1" t="inlineStr">
         <is>
           <t>lunar_phase</t>
         </is>
       </c>
-      <c r="IF1" s="1" t="inlineStr">
+      <c r="IG1" s="1" t="inlineStr">
         <is>
           <t>lunar_illumination</t>
         </is>
       </c>
-      <c r="IG1" s="1" t="inlineStr">
+      <c r="IH1" s="1" t="inlineStr">
         <is>
           <t>lunar_name</t>
         </is>
       </c>
-      <c r="IH1" s="1" t="inlineStr">
+      <c r="II1" s="1" t="inlineStr">
         <is>
           <t>monitoring_quality</t>
         </is>
@@ -2254,21 +2259,26 @@
       <c r="IC2">
         <v>1</v>
       </c>
-      <c r="ID2">
+      <c r="ID2" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE2">
         <v>5.199999999999999</v>
       </c>
-      <c r="IE2">
+      <c r="IF2">
         <v>1.152665035180047</v>
       </c>
-      <c r="IF2">
+      <c r="IG2">
         <v>0.2969732774352599</v>
       </c>
-      <c r="IG2" t="inlineStr">
+      <c r="IH2" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH2" t="inlineStr">
+      <c r="II2" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -2761,21 +2771,26 @@
       <c r="IC3">
         <v>1</v>
       </c>
-      <c r="ID3">
+      <c r="ID3" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE3">
         <v>4.4</v>
       </c>
-      <c r="IE3">
+      <c r="IF3">
         <v>1.152665035180047</v>
       </c>
-      <c r="IF3">
+      <c r="IG3">
         <v>0.2969732774352599</v>
       </c>
-      <c r="IG3" t="inlineStr">
+      <c r="IH3" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH3" t="inlineStr">
+      <c r="II3" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -3399,21 +3414,26 @@
       <c r="IC4">
         <v>0</v>
       </c>
-      <c r="ID4">
+      <c r="ID4" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE4">
         <v>3</v>
       </c>
-      <c r="IE4">
+      <c r="IF4">
         <v>1.152665035180047</v>
       </c>
-      <c r="IF4">
+      <c r="IG4">
         <v>0.2969732774352599</v>
       </c>
-      <c r="IG4" t="inlineStr">
+      <c r="IH4" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH4" t="inlineStr">
+      <c r="II4" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -3842,21 +3862,26 @@
       <c r="IC5">
         <v>0</v>
       </c>
-      <c r="ID5">
+      <c r="ID5" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE5">
         <v>3</v>
       </c>
-      <c r="IE5">
+      <c r="IF5">
         <v>1.152665035180047</v>
       </c>
-      <c r="IF5">
+      <c r="IG5">
         <v>0.2969732774352599</v>
       </c>
-      <c r="IG5" t="inlineStr">
+      <c r="IH5" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH5" t="inlineStr">
+      <c r="II5" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -4515,21 +4540,26 @@
       <c r="IC6">
         <v>1</v>
       </c>
-      <c r="ID6">
+      <c r="ID6" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE6">
         <v>2.4</v>
       </c>
-      <c r="IE6">
+      <c r="IF6">
         <v>1.152665035180047</v>
       </c>
-      <c r="IF6">
+      <c r="IG6">
         <v>0.2969732774352599</v>
       </c>
-      <c r="IG6" t="inlineStr">
+      <c r="IH6" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH6" t="inlineStr">
+      <c r="II6" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -4972,21 +5002,26 @@
       <c r="IC7">
         <v>0</v>
       </c>
-      <c r="ID7">
+      <c r="ID7" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE7">
         <v>3</v>
       </c>
-      <c r="IE7">
+      <c r="IF7">
         <v>1.152665035180047</v>
       </c>
-      <c r="IF7">
+      <c r="IG7">
         <v>0.2969732774352599</v>
       </c>
-      <c r="IG7" t="inlineStr">
+      <c r="IH7" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH7" t="inlineStr">
+      <c r="II7" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -5609,21 +5644,26 @@
       <c r="IC8">
         <v>0</v>
       </c>
-      <c r="ID8">
+      <c r="ID8" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE8">
         <v>3</v>
       </c>
-      <c r="IE8">
+      <c r="IF8">
         <v>1.152665035180047</v>
       </c>
-      <c r="IF8">
+      <c r="IG8">
         <v>0.2969732774352599</v>
       </c>
-      <c r="IG8" t="inlineStr">
+      <c r="IH8" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH8" t="inlineStr">
+      <c r="II8" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -6084,21 +6124,26 @@
       <c r="IC9">
         <v>0</v>
       </c>
-      <c r="ID9">
+      <c r="ID9" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE9">
         <v>3</v>
       </c>
-      <c r="IE9">
+      <c r="IF9">
         <v>1.152665035180047</v>
       </c>
-      <c r="IF9">
+      <c r="IG9">
         <v>0.2969732774352599</v>
       </c>
-      <c r="IG9" t="inlineStr">
+      <c r="IH9" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH9" t="inlineStr">
+      <c r="II9" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -6746,21 +6791,26 @@
       <c r="IC10">
         <v>0</v>
       </c>
-      <c r="ID10">
+      <c r="ID10" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE10">
         <v>3.35</v>
       </c>
-      <c r="IE10">
+      <c r="IF10">
         <v>1.152665035180047</v>
       </c>
-      <c r="IF10">
+      <c r="IG10">
         <v>0.2969732774352599</v>
       </c>
-      <c r="IG10" t="inlineStr">
+      <c r="IH10" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH10" t="inlineStr">
+      <c r="II10" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -7218,21 +7268,26 @@
       <c r="IC11">
         <v>1</v>
       </c>
-      <c r="ID11">
+      <c r="ID11" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE11">
         <v>5</v>
       </c>
-      <c r="IE11">
+      <c r="IF11">
         <v>1.152665035180047</v>
       </c>
-      <c r="IF11">
+      <c r="IG11">
         <v>0.2969732774352599</v>
       </c>
-      <c r="IG11" t="inlineStr">
+      <c r="IH11" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH11" t="inlineStr">
+      <c r="II11" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -7680,21 +7735,26 @@
       <c r="IC12">
         <v>0</v>
       </c>
-      <c r="ID12">
+      <c r="ID12" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE12">
         <v>6.600000000000001</v>
       </c>
-      <c r="IE12">
+      <c r="IF12">
         <v>1.790971166336796</v>
       </c>
-      <c r="IF12">
+      <c r="IG12">
         <v>0.6092001226037329</v>
       </c>
-      <c r="IG12" t="inlineStr">
+      <c r="IH12" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH12" t="inlineStr">
+      <c r="II12" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -8157,21 +8217,26 @@
       <c r="IC13">
         <v>0</v>
       </c>
-      <c r="ID13">
+      <c r="ID13" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE13">
         <v>6.2</v>
       </c>
-      <c r="IE13">
+      <c r="IF13">
         <v>1.790971166336796</v>
       </c>
-      <c r="IF13">
+      <c r="IG13">
         <v>0.6092001226037329</v>
       </c>
-      <c r="IG13" t="inlineStr">
+      <c r="IH13" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH13" t="inlineStr">
+      <c r="II13" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -8568,21 +8633,26 @@
       <c r="IC14">
         <v>0</v>
       </c>
-      <c r="ID14">
+      <c r="ID14" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE14">
         <v>3.6</v>
       </c>
-      <c r="IE14">
+      <c r="IF14">
         <v>1.578202455951332</v>
       </c>
-      <c r="IF14">
+      <c r="IG14">
         <v>0.5037030307256661</v>
       </c>
-      <c r="IG14" t="inlineStr">
+      <c r="IH14" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH14" t="inlineStr">
+      <c r="II14" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -8994,21 +9064,26 @@
       <c r="IC15">
         <v>1</v>
       </c>
-      <c r="ID15">
+      <c r="ID15" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE15">
         <v>3.5</v>
       </c>
-      <c r="IE15">
+      <c r="IF15">
         <v>1.578202455951332</v>
       </c>
-      <c r="IF15">
+      <c r="IG15">
         <v>0.5037030307256661</v>
       </c>
-      <c r="IG15" t="inlineStr">
+      <c r="IH15" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH15" t="inlineStr">
+      <c r="II15" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -9497,21 +9572,26 @@
       <c r="IC16">
         <v>1</v>
       </c>
-      <c r="ID16">
+      <c r="ID16" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE16">
         <v>5.199999999999999</v>
       </c>
-      <c r="IE16">
+      <c r="IF16">
         <v>1.578202455951332</v>
       </c>
-      <c r="IF16">
+      <c r="IG16">
         <v>0.5037030307256661</v>
       </c>
-      <c r="IG16" t="inlineStr">
+      <c r="IH16" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH16" t="inlineStr">
+      <c r="II16" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -9974,21 +10054,26 @@
       <c r="IC17">
         <v>1</v>
       </c>
-      <c r="ID17">
+      <c r="ID17" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE17">
         <v>5.199999999999999</v>
       </c>
-      <c r="IE17">
+      <c r="IF17">
         <v>1.578202455951332</v>
       </c>
-      <c r="IF17">
+      <c r="IG17">
         <v>0.5037030307256661</v>
       </c>
-      <c r="IG17" t="inlineStr">
+      <c r="IH17" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH17" t="inlineStr">
+      <c r="II17" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -10445,21 +10530,26 @@
       <c r="IC18">
         <v>1</v>
       </c>
-      <c r="ID18">
+      <c r="ID18" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE18">
         <v>5</v>
       </c>
-      <c r="IE18">
+      <c r="IF18">
         <v>1.790971166336796</v>
       </c>
-      <c r="IF18">
+      <c r="IG18">
         <v>0.6092001226037329</v>
       </c>
-      <c r="IG18" t="inlineStr">
+      <c r="IH18" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH18" t="inlineStr">
+      <c r="II18" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -10928,21 +11018,26 @@
       <c r="IC19">
         <v>1</v>
       </c>
-      <c r="ID19">
+      <c r="ID19" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE19">
         <v>6.2</v>
       </c>
-      <c r="IE19">
+      <c r="IF19">
         <v>1.790971166336796</v>
       </c>
-      <c r="IF19">
+      <c r="IG19">
         <v>0.6092001226037329</v>
       </c>
-      <c r="IG19" t="inlineStr">
+      <c r="IH19" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH19" t="inlineStr">
+      <c r="II19" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -11416,21 +11511,26 @@
       <c r="IC20">
         <v>1</v>
       </c>
-      <c r="ID20">
+      <c r="ID20" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE20">
         <v>5.699999999999999</v>
       </c>
-      <c r="IE20">
+      <c r="IF20">
         <v>1.790971166336796</v>
       </c>
-      <c r="IF20">
+      <c r="IG20">
         <v>0.6092001226037329</v>
       </c>
-      <c r="IG20" t="inlineStr">
+      <c r="IH20" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH20" t="inlineStr">
+      <c r="II20" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -11919,21 +12019,26 @@
       <c r="IC21">
         <v>1</v>
       </c>
-      <c r="ID21">
+      <c r="ID21" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE21">
         <v>5.699999999999999</v>
       </c>
-      <c r="IE21">
+      <c r="IF21">
         <v>1.790971166336796</v>
       </c>
-      <c r="IF21">
+      <c r="IG21">
         <v>0.6092001226037329</v>
       </c>
-      <c r="IG21" t="inlineStr">
+      <c r="IH21" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH21" t="inlineStr">
+      <c r="II21" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -12392,21 +12497,26 @@
       <c r="IC22">
         <v>1</v>
       </c>
-      <c r="ID22">
+      <c r="ID22" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE22">
         <v>5.557973333333334</v>
       </c>
-      <c r="IE22">
+      <c r="IF22">
         <v>0.1756807860302614</v>
       </c>
-      <c r="IF22">
+      <c r="IG22">
         <v>0.007696109834573639</v>
       </c>
-      <c r="IG22" t="inlineStr">
+      <c r="IH22" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH22" t="inlineStr">
+      <c r="II22" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -12858,21 +12968,26 @@
       <c r="IC23">
         <v>1</v>
       </c>
-      <c r="ID23">
+      <c r="ID23" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE23">
         <v>4.4</v>
       </c>
-      <c r="IE23">
+      <c r="IF23">
         <v>0.1756807860302614</v>
       </c>
-      <c r="IF23">
+      <c r="IG23">
         <v>0.007696109834573639</v>
       </c>
-      <c r="IG23" t="inlineStr">
+      <c r="IH23" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH23" t="inlineStr">
+      <c r="II23" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -13284,21 +13399,26 @@
       <c r="IC24">
         <v>0</v>
       </c>
-      <c r="ID24">
+      <c r="ID24" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE24">
         <v>3.22144</v>
       </c>
-      <c r="IE24">
+      <c r="IF24">
         <v>6.246097382824026</v>
       </c>
-      <c r="IF24">
+      <c r="IG24">
         <v>0.00034383911757635</v>
       </c>
-      <c r="IG24" t="inlineStr">
+      <c r="IH24" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH24" t="inlineStr">
+      <c r="II24" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -13746,21 +13866,26 @@
       <c r="IC25">
         <v>1</v>
       </c>
-      <c r="ID25">
+      <c r="ID25" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE25">
         <v>3</v>
       </c>
-      <c r="IE25">
+      <c r="IF25">
         <v>6.246097382824026</v>
       </c>
-      <c r="IF25">
+      <c r="IG25">
         <v>0.00034383911757635</v>
       </c>
-      <c r="IG25" t="inlineStr">
+      <c r="IH25" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH25" t="inlineStr">
+      <c r="II25" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -14203,21 +14328,26 @@
       <c r="IC26">
         <v>1</v>
       </c>
-      <c r="ID26">
+      <c r="ID26" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE26">
         <v>2.66496</v>
       </c>
-      <c r="IE26">
+      <c r="IF26">
         <v>6.246097382824026</v>
       </c>
-      <c r="IF26">
+      <c r="IG26">
         <v>0.00034383911757635</v>
       </c>
-      <c r="IG26" t="inlineStr">
+      <c r="IH26" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH26" t="inlineStr">
+      <c r="II26" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -14686,21 +14816,26 @@
       <c r="IC27">
         <v>1</v>
       </c>
-      <c r="ID27">
+      <c r="ID27" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE27">
         <v>3</v>
       </c>
-      <c r="IE27">
+      <c r="IF27">
         <v>6.246097382824026</v>
       </c>
-      <c r="IF27">
+      <c r="IG27">
         <v>0.00034383911757635</v>
       </c>
-      <c r="IG27" t="inlineStr">
+      <c r="IH27" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH27" t="inlineStr">
+      <c r="II27" t="inlineStr">
         <is>
           <t>compromised</t>
         </is>
@@ -15173,21 +15308,26 @@
       <c r="IC28">
         <v>1</v>
       </c>
-      <c r="ID28">
+      <c r="ID28" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE28">
         <v>3.203733333333333</v>
       </c>
-      <c r="IE28">
+      <c r="IF28">
         <v>6.246097382824026</v>
       </c>
-      <c r="IF28">
+      <c r="IG28">
         <v>0.00034383911757635</v>
       </c>
-      <c r="IG28" t="inlineStr">
+      <c r="IH28" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH28" t="inlineStr">
+      <c r="II28" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -15605,21 +15745,26 @@
       <c r="IC29">
         <v>0</v>
       </c>
-      <c r="ID29">
+      <c r="ID29" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE29">
         <v>3</v>
       </c>
-      <c r="IE29">
+      <c r="IF29">
         <v>6.246097382824026</v>
       </c>
-      <c r="IF29">
+      <c r="IG29">
         <v>0.00034383911757635</v>
       </c>
-      <c r="IG29" t="inlineStr">
+      <c r="IH29" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH29" t="inlineStr">
+      <c r="II29" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -16057,21 +16202,26 @@
       <c r="IC30">
         <v>1</v>
       </c>
-      <c r="ID30">
+      <c r="ID30" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE30">
         <v>3.613893333333333</v>
       </c>
-      <c r="IE30">
+      <c r="IF30">
         <v>6.246097382824026</v>
       </c>
-      <c r="IF30">
+      <c r="IG30">
         <v>0.00034383911757635</v>
       </c>
-      <c r="IG30" t="inlineStr">
+      <c r="IH30" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH30" t="inlineStr">
+      <c r="II30" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -16544,21 +16694,26 @@
       <c r="IC31">
         <v>1</v>
       </c>
-      <c r="ID31">
+      <c r="ID31" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE31">
         <v>5</v>
       </c>
-      <c r="IE31">
+      <c r="IF31">
         <v>6.246097382824026</v>
       </c>
-      <c r="IF31">
+      <c r="IG31">
         <v>0.00034383911757635</v>
       </c>
-      <c r="IG31" t="inlineStr">
+      <c r="IH31" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH31" t="inlineStr">
+      <c r="II31" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -16992,21 +17147,26 @@
       <c r="IC32">
         <v>1</v>
       </c>
-      <c r="ID32">
+      <c r="ID32" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE32">
         <v>6.600000000000001</v>
       </c>
-      <c r="IE32">
+      <c r="IF32">
         <v>0.6012182068011893</v>
       </c>
-      <c r="IF32">
+      <c r="IG32">
         <v>0.08767642431597361</v>
       </c>
-      <c r="IG32" t="inlineStr">
+      <c r="IH32" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH32" t="inlineStr">
+      <c r="II32" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -17473,21 +17633,26 @@
       <c r="IC33">
         <v>1</v>
       </c>
-      <c r="ID33">
+      <c r="ID33" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE33">
         <v>6.2</v>
       </c>
-      <c r="IE33">
+      <c r="IF33">
         <v>0.6012182068011893</v>
       </c>
-      <c r="IF33">
+      <c r="IG33">
         <v>0.08767642431597361</v>
       </c>
-      <c r="IG33" t="inlineStr">
+      <c r="IH33" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH33" t="inlineStr">
+      <c r="II33" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -17713,21 +17878,26 @@
           <t>7</t>
         </is>
       </c>
-      <c r="ID34">
+      <c r="ID34" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE34">
         <v>3.6</v>
       </c>
-      <c r="IE34">
+      <c r="IF34">
         <v>0.6012182068011893</v>
       </c>
-      <c r="IF34">
+      <c r="IG34">
         <v>0.08767642431597361</v>
       </c>
-      <c r="IG34" t="inlineStr">
+      <c r="IH34" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH34" t="inlineStr">
+      <c r="II34" t="inlineStr">
         <is>
           <t>compromised</t>
         </is>
@@ -17953,21 +18123,26 @@
           <t>7</t>
         </is>
       </c>
-      <c r="ID35">
+      <c r="ID35" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE35">
         <v>3.5</v>
       </c>
-      <c r="IE35">
+      <c r="IF35">
         <v>0.6012182068011893</v>
       </c>
-      <c r="IF35">
+      <c r="IG35">
         <v>0.08767642431597361</v>
       </c>
-      <c r="IG35" t="inlineStr">
+      <c r="IH35" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH35" t="inlineStr">
+      <c r="II35" t="inlineStr">
         <is>
           <t>compromised</t>
         </is>
@@ -18427,21 +18602,26 @@
       <c r="IC36">
         <v>1</v>
       </c>
-      <c r="ID36">
+      <c r="ID36" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE36">
         <v>5.199999999999999</v>
       </c>
-      <c r="IE36">
+      <c r="IF36">
         <v>0.6012182068011893</v>
       </c>
-      <c r="IF36">
+      <c r="IG36">
         <v>0.08767642431597361</v>
       </c>
-      <c r="IG36" t="inlineStr">
+      <c r="IH36" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH36" t="inlineStr">
+      <c r="II36" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -18905,21 +19085,26 @@
       <c r="IC37">
         <v>1</v>
       </c>
-      <c r="ID37">
+      <c r="ID37" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE37">
         <v>5.199999999999999</v>
       </c>
-      <c r="IE37">
+      <c r="IF37">
         <v>0.6012182068011893</v>
       </c>
-      <c r="IF37">
+      <c r="IG37">
         <v>0.08767642431597361</v>
       </c>
-      <c r="IG37" t="inlineStr">
+      <c r="IH37" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH37" t="inlineStr">
+      <c r="II37" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -19404,21 +19589,26 @@
       <c r="IC38">
         <v>1</v>
       </c>
-      <c r="ID38">
+      <c r="ID38" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE38">
         <v>5</v>
       </c>
-      <c r="IE38">
+      <c r="IF38">
         <v>0.6012182068011893</v>
       </c>
-      <c r="IF38">
+      <c r="IG38">
         <v>0.08767642431597361</v>
       </c>
-      <c r="IG38" t="inlineStr">
+      <c r="IH38" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH38" t="inlineStr">
+      <c r="II38" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -19927,21 +20117,26 @@
       <c r="IC39">
         <v>1</v>
       </c>
-      <c r="ID39">
+      <c r="ID39" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE39">
         <v>6.2</v>
       </c>
-      <c r="IE39">
+      <c r="IF39">
         <v>0.6012182068011893</v>
       </c>
-      <c r="IF39">
+      <c r="IG39">
         <v>0.08767642431597361</v>
       </c>
-      <c r="IG39" t="inlineStr">
+      <c r="IH39" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH39" t="inlineStr">
+      <c r="II39" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -20422,21 +20617,26 @@
       <c r="IC40">
         <v>1</v>
       </c>
-      <c r="ID40">
+      <c r="ID40" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE40">
         <v>5.699999999999999</v>
       </c>
-      <c r="IE40">
+      <c r="IF40">
         <v>0.6012182068011893</v>
       </c>
-      <c r="IF40">
+      <c r="IG40">
         <v>0.08767642431597361</v>
       </c>
-      <c r="IG40" t="inlineStr">
+      <c r="IH40" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH40" t="inlineStr">
+      <c r="II40" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -20866,21 +21066,26 @@
       <c r="IC41">
         <v>1</v>
       </c>
-      <c r="ID41">
+      <c r="ID41" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE41">
         <v>5.699999999999999</v>
       </c>
-      <c r="IE41">
+      <c r="IF41">
         <v>0.6012182068011893</v>
       </c>
-      <c r="IF41">
+      <c r="IG41">
         <v>0.08767642431597361</v>
       </c>
-      <c r="IG41" t="inlineStr">
+      <c r="IH41" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH41" t="inlineStr">
+      <c r="II41" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -21290,21 +21495,26 @@
       <c r="IC42">
         <v>0</v>
       </c>
-      <c r="ID42">
+      <c r="ID42" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE42">
         <v>5.557973333333334</v>
       </c>
-      <c r="IE42">
+      <c r="IF42">
         <v>4.418038292131671</v>
       </c>
-      <c r="IF42">
+      <c r="IG42">
         <v>0.6450592630039791</v>
       </c>
-      <c r="IG42" t="inlineStr">
+      <c r="IH42" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH42" t="inlineStr">
+      <c r="II42" t="inlineStr">
         <is>
           <t>compromised</t>
         </is>
@@ -21728,21 +21938,26 @@
       <c r="IC43">
         <v>1</v>
       </c>
-      <c r="ID43">
+      <c r="ID43" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE43">
         <v>4.4</v>
       </c>
-      <c r="IE43">
+      <c r="IF43">
         <v>4.418038292131671</v>
       </c>
-      <c r="IF43">
+      <c r="IG43">
         <v>0.6450592630039791</v>
       </c>
-      <c r="IG43" t="inlineStr">
+      <c r="IH43" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH43" t="inlineStr">
+      <c r="II43" t="inlineStr">
         <is>
           <t>compromised</t>
         </is>
@@ -22187,21 +22402,26 @@
       <c r="IC44">
         <v>0</v>
       </c>
-      <c r="ID44">
+      <c r="ID44" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE44">
         <v>3.22144</v>
       </c>
-      <c r="IE44">
+      <c r="IF44">
         <v>4.205269581746207</v>
       </c>
-      <c r="IF44">
+      <c r="IG44">
         <v>0.7428305979649599</v>
       </c>
-      <c r="IG44" t="inlineStr">
+      <c r="IH44" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH44" t="inlineStr">
+      <c r="II44" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -22646,21 +22866,26 @@
       <c r="IC45">
         <v>0</v>
       </c>
-      <c r="ID45">
+      <c r="ID45" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE45">
         <v>3</v>
       </c>
-      <c r="IE45">
+      <c r="IF45">
         <v>4.205269581746207</v>
       </c>
-      <c r="IF45">
+      <c r="IG45">
         <v>0.7428305979649599</v>
       </c>
-      <c r="IG45" t="inlineStr">
+      <c r="IH45" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH45" t="inlineStr">
+      <c r="II45" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -23061,21 +23286,26 @@
       <c r="IC46">
         <v>1</v>
       </c>
-      <c r="ID46">
+      <c r="ID46" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE46">
         <v>2.66496</v>
       </c>
-      <c r="IE46">
+      <c r="IF46">
         <v>4.205269581746207</v>
       </c>
-      <c r="IF46">
+      <c r="IG46">
         <v>0.7428305979649599</v>
       </c>
-      <c r="IG46" t="inlineStr">
+      <c r="IH46" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH46" t="inlineStr">
+      <c r="II46" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -23485,21 +23715,26 @@
       <c r="IC47">
         <v>0</v>
       </c>
-      <c r="ID47">
+      <c r="ID47" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE47">
         <v>3</v>
       </c>
-      <c r="IE47">
+      <c r="IF47">
         <v>4.205269581746207</v>
       </c>
-      <c r="IF47">
+      <c r="IG47">
         <v>0.7428305979649599</v>
       </c>
-      <c r="IG47" t="inlineStr">
+      <c r="IH47" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH47" t="inlineStr">
+      <c r="II47" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -23939,21 +24174,26 @@
       <c r="IC48">
         <v>1</v>
       </c>
-      <c r="ID48">
+      <c r="ID48" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE48">
         <v>3.203733333333333</v>
       </c>
-      <c r="IE48">
+      <c r="IF48">
         <v>4.418038292131671</v>
       </c>
-      <c r="IF48">
+      <c r="IG48">
         <v>0.6450592630039791</v>
       </c>
-      <c r="IG48" t="inlineStr">
+      <c r="IH48" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH48" t="inlineStr">
+      <c r="II48" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -24342,21 +24582,26 @@
       <c r="IC49">
         <v>0</v>
       </c>
-      <c r="ID49">
+      <c r="ID49" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE49">
         <v>3</v>
       </c>
-      <c r="IE49">
+      <c r="IF49">
         <v>4.418038292131671</v>
       </c>
-      <c r="IF49">
+      <c r="IG49">
         <v>0.6450592630039791</v>
       </c>
-      <c r="IG49" t="inlineStr">
+      <c r="IH49" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH49" t="inlineStr">
+      <c r="II49" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -24821,21 +25066,26 @@
       <c r="IC50">
         <v>1</v>
       </c>
-      <c r="ID50">
+      <c r="ID50" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE50">
         <v>3.613893333333333</v>
       </c>
-      <c r="IE50">
+      <c r="IF50">
         <v>4.205269581746207</v>
       </c>
-      <c r="IF50">
+      <c r="IG50">
         <v>0.7428305979649599</v>
       </c>
-      <c r="IG50" t="inlineStr">
+      <c r="IH50" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH50" t="inlineStr">
+      <c r="II50" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -25275,21 +25525,26 @@
       <c r="IC51">
         <v>1</v>
       </c>
-      <c r="ID51">
+      <c r="ID51" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE51">
         <v>5</v>
       </c>
-      <c r="IE51">
+      <c r="IF51">
         <v>4.205269581746207</v>
       </c>
-      <c r="IF51">
+      <c r="IG51">
         <v>0.7428305979649599</v>
       </c>
-      <c r="IG51" t="inlineStr">
+      <c r="IH51" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH51" t="inlineStr">
+      <c r="II51" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -25759,21 +26014,26 @@
       <c r="IC52">
         <v>0</v>
       </c>
-      <c r="ID52">
+      <c r="ID52" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE52">
         <v>6.600000000000001</v>
       </c>
-      <c r="IE52">
+      <c r="IF52">
         <v>1.32638364073583</v>
       </c>
-      <c r="IF52">
+      <c r="IG52">
         <v>0.3790067460938265</v>
       </c>
-      <c r="IG52" t="inlineStr">
+      <c r="IH52" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH52" t="inlineStr">
+      <c r="II52" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -26237,21 +26497,26 @@
       <c r="IC53">
         <v>1</v>
       </c>
-      <c r="ID53">
+      <c r="ID53" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE53">
         <v>6.2</v>
       </c>
-      <c r="IE53">
+      <c r="IF53">
         <v>1.113614930350366</v>
       </c>
-      <c r="IF53">
+      <c r="IG53">
         <v>0.2792896349616143</v>
       </c>
-      <c r="IG53" t="inlineStr">
+      <c r="IH53" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH53" t="inlineStr">
+      <c r="II53" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -26694,21 +26959,26 @@
       <c r="IC54">
         <v>1</v>
       </c>
-      <c r="ID54">
+      <c r="ID54" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE54">
         <v>3.6</v>
       </c>
-      <c r="IE54">
+      <c r="IF54">
         <v>1.113614930350366</v>
       </c>
-      <c r="IF54">
+      <c r="IG54">
         <v>0.2792896349616143</v>
       </c>
-      <c r="IG54" t="inlineStr">
+      <c r="IH54" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH54" t="inlineStr">
+      <c r="II54" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -27156,21 +27426,26 @@
       <c r="IC55">
         <v>0</v>
       </c>
-      <c r="ID55">
+      <c r="ID55" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE55">
         <v>3.5</v>
       </c>
-      <c r="IE55">
+      <c r="IF55">
         <v>1.113614930350366</v>
       </c>
-      <c r="IF55">
+      <c r="IG55">
         <v>0.2792896349616143</v>
       </c>
-      <c r="IG55" t="inlineStr">
+      <c r="IH55" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH55" t="inlineStr">
+      <c r="II55" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -27618,21 +27893,26 @@
       <c r="IC56">
         <v>1</v>
       </c>
-      <c r="ID56">
+      <c r="ID56" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE56">
         <v>5.199999999999999</v>
       </c>
-      <c r="IE56">
+      <c r="IF56">
         <v>1.113614930350366</v>
       </c>
-      <c r="IF56">
+      <c r="IG56">
         <v>0.2792896349616143</v>
       </c>
-      <c r="IG56" t="inlineStr">
+      <c r="IH56" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH56" t="inlineStr">
+      <c r="II56" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -28015,21 +28295,26 @@
       <c r="IC57">
         <v>0</v>
       </c>
-      <c r="ID57">
+      <c r="ID57" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE57">
         <v>5.199999999999999</v>
       </c>
-      <c r="IE57">
+      <c r="IF57">
         <v>1.113614930350366</v>
       </c>
-      <c r="IF57">
+      <c r="IG57">
         <v>0.2792896349616143</v>
       </c>
-      <c r="IG57" t="inlineStr">
+      <c r="IH57" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH57" t="inlineStr">
+      <c r="II57" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -28502,21 +28787,26 @@
       <c r="IC58">
         <v>1</v>
       </c>
-      <c r="ID58">
+      <c r="ID58" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE58">
         <v>5</v>
       </c>
-      <c r="IE58">
+      <c r="IF58">
         <v>1.113614930350366</v>
       </c>
-      <c r="IF58">
+      <c r="IG58">
         <v>0.2792896349616143</v>
       </c>
-      <c r="IG58" t="inlineStr">
+      <c r="IH58" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH58" t="inlineStr">
+      <c r="II58" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -28959,21 +29249,26 @@
       <c r="IC59">
         <v>0</v>
       </c>
-      <c r="ID59">
+      <c r="ID59" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE59">
         <v>6.2</v>
       </c>
-      <c r="IE59">
+      <c r="IF59">
         <v>1.113614930350366</v>
       </c>
-      <c r="IF59">
+      <c r="IG59">
         <v>0.2792896349616143</v>
       </c>
-      <c r="IG59" t="inlineStr">
+      <c r="IH59" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH59" t="inlineStr">
+      <c r="II59" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -29426,21 +29721,26 @@
       <c r="IC60">
         <v>1</v>
       </c>
-      <c r="ID60">
+      <c r="ID60" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE60">
         <v>5.699999999999999</v>
       </c>
-      <c r="IE60">
+      <c r="IF60">
         <v>1.113614930350366</v>
       </c>
-      <c r="IF60">
+      <c r="IG60">
         <v>0.2792896349616143</v>
       </c>
-      <c r="IG60" t="inlineStr">
+      <c r="IH60" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH60" t="inlineStr">
+      <c r="II60" t="inlineStr">
         <is>
           <t>compromised</t>
         </is>
@@ -29884,21 +30184,26 @@
       <c r="IC61">
         <v>1</v>
       </c>
-      <c r="ID61">
+      <c r="ID61" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE61">
         <v>5.699999999999999</v>
       </c>
-      <c r="IE61">
+      <c r="IF61">
         <v>1.113614930350366</v>
       </c>
-      <c r="IF61">
+      <c r="IG61">
         <v>0.2792896349616143</v>
       </c>
-      <c r="IG61" t="inlineStr">
+      <c r="IH61" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH61" t="inlineStr">
+      <c r="II61" t="inlineStr">
         <is>
           <t>compromised</t>
         </is>
@@ -30116,21 +30421,26 @@
           <t>1</t>
         </is>
       </c>
-      <c r="ID62">
+      <c r="ID62" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE62">
         <v>5.557973333333334</v>
       </c>
-      <c r="IE62">
+      <c r="IF62">
         <v>5.994278567608524</v>
       </c>
-      <c r="IF62">
+      <c r="IG62">
         <v>0.02072203847629311</v>
       </c>
-      <c r="IG62" t="inlineStr">
+      <c r="IH62" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH62" t="inlineStr">
+      <c r="II62" t="inlineStr">
         <is>
           <t>compromised</t>
         </is>
@@ -30353,21 +30663,26 @@
           <t>1</t>
         </is>
       </c>
-      <c r="ID63">
+      <c r="ID63" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE63">
         <v>4.4</v>
       </c>
-      <c r="IE63">
+      <c r="IF63">
         <v>6.207047277994345</v>
       </c>
-      <c r="IF63">
+      <c r="IG63">
         <v>0.001448549898926232</v>
       </c>
-      <c r="IG63" t="inlineStr">
+      <c r="IH63" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH63" t="inlineStr">
+      <c r="II63" t="inlineStr">
         <is>
           <t>compromised</t>
         </is>
@@ -30767,21 +31082,26 @@
       <c r="IC64">
         <v>0</v>
       </c>
-      <c r="ID64">
+      <c r="ID64" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE64">
         <v>3.22144</v>
       </c>
-      <c r="IE64">
+      <c r="IF64">
         <v>5.994278567608524</v>
       </c>
-      <c r="IF64">
+      <c r="IG64">
         <v>0.02072203847629311</v>
       </c>
-      <c r="IG64" t="inlineStr">
+      <c r="IH64" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH64" t="inlineStr">
+      <c r="II64" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -31202,21 +31522,26 @@
       <c r="IC65">
         <v>0</v>
       </c>
-      <c r="ID65">
+      <c r="ID65" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE65">
         <v>3</v>
       </c>
-      <c r="IE65">
+      <c r="IF65">
         <v>5.994278567608524</v>
       </c>
-      <c r="IF65">
+      <c r="IG65">
         <v>0.02072203847629311</v>
       </c>
-      <c r="IG65" t="inlineStr">
+      <c r="IH65" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH65" t="inlineStr">
+      <c r="II65" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -31650,21 +31975,26 @@
       <c r="IC66">
         <v>1</v>
       </c>
-      <c r="ID66">
+      <c r="ID66" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE66">
         <v>2.66496</v>
       </c>
-      <c r="IE66">
+      <c r="IF66">
         <v>5.994278567608524</v>
       </c>
-      <c r="IF66">
+      <c r="IG66">
         <v>0.02072203847629311</v>
       </c>
-      <c r="IG66" t="inlineStr">
+      <c r="IH66" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH66" t="inlineStr">
+      <c r="II66" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -32122,21 +32452,26 @@
       <c r="IC67">
         <v>1</v>
       </c>
-      <c r="ID67">
+      <c r="ID67" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE67">
         <v>3</v>
       </c>
-      <c r="IE67">
+      <c r="IF67">
         <v>5.994278567608524</v>
       </c>
-      <c r="IF67">
+      <c r="IG67">
         <v>0.02072203847629311</v>
       </c>
-      <c r="IG67" t="inlineStr">
+      <c r="IH67" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH67" t="inlineStr">
+      <c r="II67" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -32570,21 +32905,26 @@
       <c r="IC68">
         <v>1</v>
       </c>
-      <c r="ID68">
+      <c r="ID68" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE68">
         <v>3.203733333333333</v>
       </c>
-      <c r="IE68">
+      <c r="IF68">
         <v>5.994278567608524</v>
       </c>
-      <c r="IF68">
+      <c r="IG68">
         <v>0.02072203847629311</v>
       </c>
-      <c r="IG68" t="inlineStr">
+      <c r="IH68" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH68" t="inlineStr">
+      <c r="II68" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -32976,21 +33316,26 @@
       <c r="IC69">
         <v>0</v>
       </c>
-      <c r="ID69">
+      <c r="ID69" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE69">
         <v>3</v>
       </c>
-      <c r="IE69">
+      <c r="IF69">
         <v>5.994278567608524</v>
       </c>
-      <c r="IF69">
+      <c r="IG69">
         <v>0.02072203847629311</v>
       </c>
-      <c r="IG69" t="inlineStr">
+      <c r="IH69" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH69" t="inlineStr">
+      <c r="II69" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -33419,21 +33764,26 @@
       <c r="IC70">
         <v>1</v>
       </c>
-      <c r="ID70">
+      <c r="ID70" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE70">
         <v>3.613893333333333</v>
       </c>
-      <c r="IE70">
+      <c r="IF70">
         <v>5.994278567608524</v>
       </c>
-      <c r="IF70">
+      <c r="IG70">
         <v>0.02072203847629311</v>
       </c>
-      <c r="IG70" t="inlineStr">
+      <c r="IH70" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH70" t="inlineStr">
+      <c r="II70" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -33846,21 +34196,26 @@
       <c r="IC71">
         <v>1</v>
       </c>
-      <c r="ID71">
+      <c r="ID71" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE71">
         <v>5</v>
       </c>
-      <c r="IE71">
+      <c r="IF71">
         <v>5.994278567608524</v>
       </c>
-      <c r="IF71">
+      <c r="IG71">
         <v>0.02072203847629311</v>
       </c>
-      <c r="IG71" t="inlineStr">
+      <c r="IH71" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH71" t="inlineStr">
+      <c r="II71" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -34354,21 +34709,26 @@
       <c r="IC72">
         <v>1</v>
       </c>
-      <c r="ID72">
+      <c r="ID72" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE72">
         <v>6.600000000000001</v>
       </c>
-      <c r="IE72">
+      <c r="IF72">
         <v>3.966467468140717</v>
       </c>
-      <c r="IF72">
+      <c r="IG72">
         <v>0.83932445750031</v>
       </c>
-      <c r="IG72" t="inlineStr">
+      <c r="IH72" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH72" t="inlineStr">
+      <c r="II72" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -34841,21 +35201,26 @@
       <c r="IC73">
         <v>0</v>
       </c>
-      <c r="ID73">
+      <c r="ID73" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE73">
         <v>6.2</v>
       </c>
-      <c r="IE73">
+      <c r="IF73">
         <v>3.966467468140717</v>
       </c>
-      <c r="IF73">
+      <c r="IG73">
         <v>0.83932445750031</v>
       </c>
-      <c r="IG73" t="inlineStr">
+      <c r="IH73" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH73" t="inlineStr">
+      <c r="II73" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -35289,21 +35654,26 @@
       <c r="IC74">
         <v>0</v>
       </c>
-      <c r="ID74">
+      <c r="ID74" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE74">
         <v>3.6</v>
       </c>
-      <c r="IE74">
+      <c r="IF74">
         <v>3.966467468140717</v>
       </c>
-      <c r="IF74">
+      <c r="IG74">
         <v>0.83932445750031</v>
       </c>
-      <c r="IG74" t="inlineStr">
+      <c r="IH74" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH74" t="inlineStr">
+      <c r="II74" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -35725,21 +36095,26 @@
       <c r="IC75">
         <v>0</v>
       </c>
-      <c r="ID75">
+      <c r="ID75" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE75">
         <v>3.5</v>
       </c>
-      <c r="IE75">
+      <c r="IF75">
         <v>3.966467468140717</v>
       </c>
-      <c r="IF75">
+      <c r="IG75">
         <v>0.83932445750031</v>
       </c>
-      <c r="IG75" t="inlineStr">
+      <c r="IH75" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH75" t="inlineStr">
+      <c r="II75" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -36178,21 +36553,26 @@
       <c r="IC76">
         <v>1</v>
       </c>
-      <c r="ID76">
+      <c r="ID76" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE76">
         <v>5.199999999999999</v>
       </c>
-      <c r="IE76">
+      <c r="IF76">
         <v>3.966467468140717</v>
       </c>
-      <c r="IF76">
+      <c r="IG76">
         <v>0.83932445750031</v>
       </c>
-      <c r="IG76" t="inlineStr">
+      <c r="IH76" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH76" t="inlineStr">
+      <c r="II76" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -36626,21 +37006,26 @@
       <c r="IC77">
         <v>1</v>
       </c>
-      <c r="ID77">
+      <c r="ID77" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE77">
         <v>5.199999999999999</v>
       </c>
-      <c r="IE77">
+      <c r="IF77">
         <v>3.966467468140717</v>
       </c>
-      <c r="IF77">
+      <c r="IG77">
         <v>0.83932445750031</v>
       </c>
-      <c r="IG77" t="inlineStr">
+      <c r="IH77" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH77" t="inlineStr">
+      <c r="II77" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -37134,21 +37519,26 @@
       <c r="IC78">
         <v>1</v>
       </c>
-      <c r="ID78">
+      <c r="ID78" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE78">
         <v>5</v>
       </c>
-      <c r="IE78">
+      <c r="IF78">
         <v>3.966467468140717</v>
       </c>
-      <c r="IF78">
+      <c r="IG78">
         <v>0.83932445750031</v>
       </c>
-      <c r="IG78" t="inlineStr">
+      <c r="IH78" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH78" t="inlineStr">
+      <c r="II78" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -37570,21 +37960,26 @@
       <c r="IC79">
         <v>1</v>
       </c>
-      <c r="ID79">
+      <c r="ID79" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE79">
         <v>6.2</v>
       </c>
-      <c r="IE79">
+      <c r="IF79">
         <v>3.966467468140717</v>
       </c>
-      <c r="IF79">
+      <c r="IG79">
         <v>0.83932445750031</v>
       </c>
-      <c r="IG79" t="inlineStr">
+      <c r="IH79" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH79" t="inlineStr">
+      <c r="II79" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -38032,21 +38427,26 @@
       <c r="IC80">
         <v>1</v>
       </c>
-      <c r="ID80">
+      <c r="ID80" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE80">
         <v>5.699999999999999</v>
       </c>
-      <c r="IE80">
+      <c r="IF80">
         <v>3.966467468140717</v>
       </c>
-      <c r="IF80">
+      <c r="IG80">
         <v>0.83932445750031</v>
       </c>
-      <c r="IG80" t="inlineStr">
+      <c r="IH80" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH80" t="inlineStr">
+      <c r="II80" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -38494,21 +38894,26 @@
       <c r="IC81">
         <v>1</v>
       </c>
-      <c r="ID81">
+      <c r="ID81" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE81">
         <v>5.699999999999999</v>
       </c>
-      <c r="IE81">
+      <c r="IF81">
         <v>3.966467468140717</v>
       </c>
-      <c r="IF81">
+      <c r="IG81">
         <v>0.83932445750031</v>
       </c>
-      <c r="IG81" t="inlineStr">
+      <c r="IH81" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH81" t="inlineStr">
+      <c r="II81" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -38958,21 +39363,26 @@
       <c r="IC82">
         <v>1</v>
       </c>
-      <c r="ID82">
+      <c r="ID82" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE82">
         <v>5.557973333333334</v>
       </c>
-      <c r="IE82">
+      <c r="IF82">
         <v>4.804525608072918</v>
       </c>
-      <c r="IF82">
+      <c r="IG82">
         <v>0.453996838695637</v>
       </c>
-      <c r="IG82" t="inlineStr">
+      <c r="IH82" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH82" t="inlineStr">
+      <c r="II82" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -39418,21 +39828,26 @@
       <c r="IC83">
         <v>1</v>
       </c>
-      <c r="ID83">
+      <c r="ID83" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE83">
         <v>4.4</v>
       </c>
-      <c r="IE83">
+      <c r="IF83">
         <v>4.804525608072918</v>
       </c>
-      <c r="IF83">
+      <c r="IG83">
         <v>0.453996838695637</v>
       </c>
-      <c r="IG83" t="inlineStr">
+      <c r="IH83" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH83" t="inlineStr">
+      <c r="II83" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -39832,21 +40247,26 @@
       <c r="IC84">
         <v>0</v>
       </c>
-      <c r="ID84">
+      <c r="ID84" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE84">
         <v>3.22144</v>
       </c>
-      <c r="IE84">
+      <c r="IF84">
         <v>4.804525608072918</v>
       </c>
-      <c r="IF84">
+      <c r="IG84">
         <v>0.453996838695637</v>
       </c>
-      <c r="IG84" t="inlineStr">
+      <c r="IH84" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH84" t="inlineStr">
+      <c r="II84" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -40267,21 +40687,26 @@
       <c r="IC85">
         <v>0</v>
       </c>
-      <c r="ID85">
+      <c r="ID85" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE85">
         <v>3</v>
       </c>
-      <c r="IE85">
+      <c r="IF85">
         <v>4.804525608072918</v>
       </c>
-      <c r="IF85">
+      <c r="IG85">
         <v>0.453996838695637</v>
       </c>
-      <c r="IG85" t="inlineStr">
+      <c r="IH85" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH85" t="inlineStr">
+      <c r="II85" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -40742,21 +41167,26 @@
       <c r="IC86">
         <v>1</v>
       </c>
-      <c r="ID86">
+      <c r="ID86" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE86">
         <v>2.66496</v>
       </c>
-      <c r="IE86">
+      <c r="IF86">
         <v>4.804525608072918</v>
       </c>
-      <c r="IF86">
+      <c r="IG86">
         <v>0.453996838695637</v>
       </c>
-      <c r="IG86" t="inlineStr">
+      <c r="IH86" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH86" t="inlineStr">
+      <c r="II86" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -41217,21 +41647,26 @@
       <c r="IC87">
         <v>1</v>
       </c>
-      <c r="ID87">
+      <c r="ID87" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE87">
         <v>3</v>
       </c>
-      <c r="IE87">
+      <c r="IF87">
         <v>4.804525608072918</v>
       </c>
-      <c r="IF87">
+      <c r="IG87">
         <v>0.453996838695637</v>
       </c>
-      <c r="IG87" t="inlineStr">
+      <c r="IH87" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH87" t="inlineStr">
+      <c r="II87" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -41722,21 +42157,26 @@
       <c r="IC88">
         <v>1</v>
       </c>
-      <c r="ID88">
+      <c r="ID88" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE88">
         <v>3.203733333333333</v>
       </c>
-      <c r="IE88">
+      <c r="IF88">
         <v>0.01072127359265074</v>
       </c>
-      <c r="IF88">
+      <c r="IG88">
         <v>2.873615160242649E-05</v>
       </c>
-      <c r="IG88" t="inlineStr">
+      <c r="IH88" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH88" t="inlineStr">
+      <c r="II88" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -42161,21 +42601,26 @@
       <c r="IC89">
         <v>0</v>
       </c>
-      <c r="ID89">
+      <c r="ID89" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE89">
         <v>3</v>
       </c>
-      <c r="IE89">
+      <c r="IF89">
         <v>0.01072127359265074</v>
       </c>
-      <c r="IF89">
+      <c r="IG89">
         <v>2.873615160242649E-05</v>
       </c>
-      <c r="IG89" t="inlineStr">
+      <c r="IH89" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH89" t="inlineStr">
+      <c r="II89" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -42610,21 +43055,26 @@
       <c r="IC90">
         <v>1</v>
       </c>
-      <c r="ID90">
+      <c r="ID90" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE90">
         <v>3.613893333333333</v>
       </c>
-      <c r="IE90">
+      <c r="IF90">
         <v>4.804525608072918</v>
       </c>
-      <c r="IF90">
+      <c r="IG90">
         <v>0.453996838695637</v>
       </c>
-      <c r="IG90" t="inlineStr">
+      <c r="IH90" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH90" t="inlineStr">
+      <c r="II90" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -43070,21 +43520,26 @@
       <c r="IC91">
         <v>1</v>
       </c>
-      <c r="ID91">
+      <c r="ID91" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE91">
         <v>5</v>
       </c>
-      <c r="IE91">
+      <c r="IF91">
         <v>4.804525608072918</v>
       </c>
-      <c r="IF91">
+      <c r="IG91">
         <v>0.453996838695637</v>
       </c>
-      <c r="IG91" t="inlineStr">
+      <c r="IH91" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH91" t="inlineStr">
+      <c r="II91" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -43548,21 +44003,26 @@
       <c r="IC92">
         <v>1</v>
       </c>
-      <c r="ID92">
+      <c r="ID92" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE92">
         <v>6.600000000000001</v>
       </c>
-      <c r="IE92">
+      <c r="IF92">
         <v>5.230063028844203</v>
       </c>
-      <c r="IF92">
+      <c r="IG92">
         <v>0.2525698548833967</v>
       </c>
-      <c r="IG92" t="inlineStr">
+      <c r="IH92" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH92" t="inlineStr">
+      <c r="II92" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -44056,21 +44516,26 @@
       <c r="IC93">
         <v>1</v>
       </c>
-      <c r="ID93">
+      <c r="ID93" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE93">
         <v>6.2</v>
       </c>
-      <c r="IE93">
+      <c r="IF93">
         <v>5.230063028844203</v>
       </c>
-      <c r="IF93">
+      <c r="IG93">
         <v>0.2525698548833967</v>
       </c>
-      <c r="IG93" t="inlineStr">
+      <c r="IH93" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH93" t="inlineStr">
+      <c r="II93" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -44492,21 +44957,26 @@
       <c r="IC94">
         <v>0</v>
       </c>
-      <c r="ID94">
+      <c r="ID94" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE94">
         <v>3.6</v>
       </c>
-      <c r="IE94">
+      <c r="IF94">
         <v>5.230063028844203</v>
       </c>
-      <c r="IF94">
+      <c r="IG94">
         <v>0.2525698548833967</v>
       </c>
-      <c r="IG94" t="inlineStr">
+      <c r="IH94" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH94" t="inlineStr">
+      <c r="II94" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -44928,21 +45398,26 @@
       <c r="IC95">
         <v>1</v>
       </c>
-      <c r="ID95">
+      <c r="ID95" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE95">
         <v>3.5</v>
       </c>
-      <c r="IE95">
+      <c r="IF95">
         <v>5.230063028844203</v>
       </c>
-      <c r="IF95">
+      <c r="IG95">
         <v>0.2525698548833967</v>
       </c>
-      <c r="IG95" t="inlineStr">
+      <c r="IH95" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH95" t="inlineStr">
+      <c r="II95" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -45390,21 +45865,26 @@
       <c r="IC96">
         <v>1</v>
       </c>
-      <c r="ID96">
+      <c r="ID96" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE96">
         <v>5.199999999999999</v>
       </c>
-      <c r="IE96">
+      <c r="IF96">
         <v>5.230063028844203</v>
       </c>
-      <c r="IF96">
+      <c r="IG96">
         <v>0.2525698548833967</v>
       </c>
-      <c r="IG96" t="inlineStr">
+      <c r="IH96" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH96" t="inlineStr">
+      <c r="II96" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -45913,21 +46393,26 @@
       <c r="IC97">
         <v>1</v>
       </c>
-      <c r="ID97">
+      <c r="ID97" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE97">
         <v>5.199999999999999</v>
       </c>
-      <c r="IE97">
+      <c r="IF97">
         <v>5.230063028844203</v>
       </c>
-      <c r="IF97">
+      <c r="IG97">
         <v>0.2525698548833967</v>
       </c>
-      <c r="IG97" t="inlineStr">
+      <c r="IH97" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH97" t="inlineStr">
+      <c r="II97" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -46379,21 +46864,26 @@
       <c r="IC98">
         <v>1</v>
       </c>
-      <c r="ID98">
+      <c r="ID98" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE98">
         <v>5</v>
       </c>
-      <c r="IE98">
+      <c r="IF98">
         <v>5.230063028844203</v>
       </c>
-      <c r="IF98">
+      <c r="IG98">
         <v>0.2525698548833967</v>
       </c>
-      <c r="IG98" t="inlineStr">
+      <c r="IH98" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH98" t="inlineStr">
+      <c r="II98" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -46845,21 +47335,26 @@
       <c r="IC99">
         <v>1</v>
       </c>
-      <c r="ID99">
+      <c r="ID99" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE99">
         <v>6.2</v>
       </c>
-      <c r="IE99">
+      <c r="IF99">
         <v>5.230063028844203</v>
       </c>
-      <c r="IF99">
+      <c r="IG99">
         <v>0.2525698548833967</v>
       </c>
-      <c r="IG99" t="inlineStr">
+      <c r="IH99" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH99" t="inlineStr">
+      <c r="II99" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -47298,21 +47793,26 @@
       <c r="IC100">
         <v>1</v>
       </c>
-      <c r="ID100">
+      <c r="ID100" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE100">
         <v>5.699999999999999</v>
       </c>
-      <c r="IE100">
+      <c r="IF100">
         <v>5.230063028844203</v>
       </c>
-      <c r="IF100">
+      <c r="IG100">
         <v>0.2525698548833967</v>
       </c>
-      <c r="IG100" t="inlineStr">
+      <c r="IH100" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH100" t="inlineStr">
+      <c r="II100" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -47721,21 +48221,26 @@
       <c r="IC101">
         <v>1</v>
       </c>
-      <c r="ID101">
+      <c r="ID101" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE101">
         <v>5.699999999999999</v>
       </c>
-      <c r="IE101">
+      <c r="IF101">
         <v>5.230063028844203</v>
       </c>
-      <c r="IF101">
+      <c r="IG101">
         <v>0.2525698548833967</v>
       </c>
-      <c r="IG101" t="inlineStr">
+      <c r="IH101" t="inlineStr">
         <is>
           <t>Waning</t>
         </is>
       </c>
-      <c r="IH101" t="inlineStr">
+      <c r="II101" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -48161,21 +48666,26 @@
       <c r="IC102">
         <v>1</v>
       </c>
-      <c r="ID102">
+      <c r="ID102" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE102">
         <v>5.557973333333334</v>
       </c>
-      <c r="IE102">
+      <c r="IF102">
         <v>1.161424128298219</v>
       </c>
-      <c r="IF102">
+      <c r="IG102">
         <v>0.3009832601809674</v>
       </c>
-      <c r="IG102" t="inlineStr">
+      <c r="IH102" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH102" t="inlineStr">
+      <c r="II102" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -48591,21 +49101,26 @@
       <c r="IC103">
         <v>0</v>
       </c>
-      <c r="ID103">
+      <c r="ID103" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE103">
         <v>4.4</v>
       </c>
-      <c r="IE103">
+      <c r="IF103">
         <v>1.161424128298219</v>
       </c>
-      <c r="IF103">
+      <c r="IG103">
         <v>0.3009832601809674</v>
       </c>
-      <c r="IG103" t="inlineStr">
+      <c r="IH103" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH103" t="inlineStr">
+      <c r="II103" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -49071,21 +49586,26 @@
       <c r="IC104">
         <v>1</v>
       </c>
-      <c r="ID104">
+      <c r="ID104" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE104">
         <v>3.22144</v>
       </c>
-      <c r="IE104">
+      <c r="IF104">
         <v>1.161424128298219</v>
       </c>
-      <c r="IF104">
+      <c r="IG104">
         <v>0.3009832601809674</v>
       </c>
-      <c r="IG104" t="inlineStr">
+      <c r="IH104" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH104" t="inlineStr">
+      <c r="II104" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -49521,21 +50041,26 @@
       <c r="IC105">
         <v>1</v>
       </c>
-      <c r="ID105">
+      <c r="ID105" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE105">
         <v>3</v>
       </c>
-      <c r="IE105">
+      <c r="IF105">
         <v>1.161424128298219</v>
       </c>
-      <c r="IF105">
+      <c r="IG105">
         <v>0.3009832601809674</v>
       </c>
-      <c r="IG105" t="inlineStr">
+      <c r="IH105" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH105" t="inlineStr">
+      <c r="II105" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -49996,21 +50521,26 @@
       <c r="IC106">
         <v>1</v>
       </c>
-      <c r="ID106">
+      <c r="ID106" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE106">
         <v>2.66496</v>
       </c>
-      <c r="IE106">
+      <c r="IF106">
         <v>0.9486554179127552</v>
       </c>
-      <c r="IF106">
+      <c r="IG106">
         <v>0.2086118663805391</v>
       </c>
-      <c r="IG106" t="inlineStr">
+      <c r="IH106" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH106" t="inlineStr">
+      <c r="II106" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -50416,21 +50946,26 @@
       <c r="IC107">
         <v>0</v>
       </c>
-      <c r="ID107">
+      <c r="ID107" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE107">
         <v>3</v>
       </c>
-      <c r="IE107">
+      <c r="IF107">
         <v>0.9486554179127552</v>
       </c>
-      <c r="IF107">
+      <c r="IG107">
         <v>0.2086118663805391</v>
       </c>
-      <c r="IG107" t="inlineStr">
+      <c r="IH107" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH107" t="inlineStr">
+      <c r="II107" t="inlineStr">
         <is>
           <t>compromised</t>
         </is>
@@ -50891,21 +51426,26 @@
       <c r="IC108">
         <v>1</v>
       </c>
-      <c r="ID108">
+      <c r="ID108" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE108">
         <v>3.203733333333333</v>
       </c>
-      <c r="IE108">
+      <c r="IF108">
         <v>1.161424128298219</v>
       </c>
-      <c r="IF108">
+      <c r="IG108">
         <v>0.3009832601809674</v>
       </c>
-      <c r="IG108" t="inlineStr">
+      <c r="IH108" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH108" t="inlineStr">
+      <c r="II108" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -51300,21 +51840,26 @@
       <c r="IC109">
         <v>0</v>
       </c>
-      <c r="ID109">
+      <c r="ID109" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE109">
         <v>3</v>
       </c>
-      <c r="IE109">
+      <c r="IF109">
         <v>1.161424128298219</v>
       </c>
-      <c r="IF109">
+      <c r="IG109">
         <v>0.3009832601809674</v>
       </c>
-      <c r="IG109" t="inlineStr">
+      <c r="IH109" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH109" t="inlineStr">
+      <c r="II109" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -51770,21 +52315,26 @@
       <c r="IC110">
         <v>1</v>
       </c>
-      <c r="ID110">
+      <c r="ID110" t="inlineStr">
+        <is>
+          <t>Stone_pile</t>
+        </is>
+      </c>
+      <c r="IE110">
         <v>3.613893333333333</v>
       </c>
-      <c r="IE110">
+      <c r="IF110">
         <v>0.9486554179127552</v>
       </c>
-      <c r="IF110">
+      <c r="IG110">
         <v>0.2086118663805391</v>
       </c>
-      <c r="IG110" t="inlineStr">
+      <c r="IH110" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH110" t="inlineStr">
+      <c r="II110" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -52215,21 +52765,26 @@
       <c r="IC111">
         <v>1</v>
       </c>
-      <c r="ID111">
+      <c r="ID111" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="IE111">
         <v>5</v>
       </c>
-      <c r="IE111">
+      <c r="IF111">
         <v>0.9486554179127552</v>
       </c>
-      <c r="IF111">
+      <c r="IG111">
         <v>0.2086118663805391</v>
       </c>
-      <c r="IG111" t="inlineStr">
+      <c r="IH111" t="inlineStr">
         <is>
           <t>Waxing</t>
         </is>
       </c>
-      <c r="IH111" t="inlineStr">
+      <c r="II111" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -52732,21 +53287,26 @@
       <c r="IC112">
         <v>1</v>
       </c>
-      <c r="ID112">
+      <c r="ID112" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE112">
         <v>6.600000000000001</v>
       </c>
-      <c r="IE112">
+      <c r="IF112">
         <v>0.7358867075269341</v>
       </c>
-      <c r="IF112">
+      <c r="IG112">
         <v>0.1293820764152031</v>
       </c>
-      <c r="IG112" t="inlineStr">
+      <c r="IH112" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH112" t="inlineStr">
+      <c r="II112" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -53219,21 +53779,26 @@
       <c r="IC113">
         <v>1</v>
       </c>
-      <c r="ID113">
+      <c r="ID113" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE113">
         <v>6.2</v>
       </c>
-      <c r="IE113">
+      <c r="IF113">
         <v>0.7358867075269341</v>
       </c>
-      <c r="IF113">
+      <c r="IG113">
         <v>0.1293820764152031</v>
       </c>
-      <c r="IG113" t="inlineStr">
+      <c r="IH113" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH113" t="inlineStr">
+      <c r="II113" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -53637,21 +54202,26 @@
       <c r="IC114">
         <v>0</v>
       </c>
-      <c r="ID114">
+      <c r="ID114" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE114">
         <v>3.6</v>
       </c>
-      <c r="IE114">
+      <c r="IF114">
         <v>0.7358867075269341</v>
       </c>
-      <c r="IF114">
+      <c r="IG114">
         <v>0.1293820764152031</v>
       </c>
-      <c r="IG114" t="inlineStr">
+      <c r="IH114" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH114" t="inlineStr">
+      <c r="II114" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -54055,21 +54625,26 @@
       <c r="IC115">
         <v>0</v>
       </c>
-      <c r="ID115">
+      <c r="ID115" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE115">
         <v>3.5</v>
       </c>
-      <c r="IE115">
+      <c r="IF115">
         <v>0.7358867075269341</v>
       </c>
-      <c r="IF115">
+      <c r="IG115">
         <v>0.1293820764152031</v>
       </c>
-      <c r="IG115" t="inlineStr">
+      <c r="IH115" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH115" t="inlineStr">
+      <c r="II115" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -54538,21 +55113,26 @@
       <c r="IC116">
         <v>1</v>
       </c>
-      <c r="ID116">
+      <c r="ID116" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE116">
         <v>5.199999999999999</v>
       </c>
-      <c r="IE116">
+      <c r="IF116">
         <v>0.7358867075269341</v>
       </c>
-      <c r="IF116">
+      <c r="IG116">
         <v>0.1293820764152031</v>
       </c>
-      <c r="IG116" t="inlineStr">
+      <c r="IH116" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH116" t="inlineStr">
+      <c r="II116" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -55016,21 +55596,26 @@
       <c r="IC117">
         <v>0</v>
       </c>
-      <c r="ID117">
+      <c r="ID117" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE117">
         <v>5.199999999999999</v>
       </c>
-      <c r="IE117">
+      <c r="IF117">
         <v>0.7358867075269341</v>
       </c>
-      <c r="IF117">
+      <c r="IG117">
         <v>0.1293820764152031</v>
       </c>
-      <c r="IG117" t="inlineStr">
+      <c r="IH117" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH117" t="inlineStr">
+      <c r="II117" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -55506,21 +56091,26 @@
       <c r="IC118">
         <v>1</v>
       </c>
-      <c r="ID118">
+      <c r="ID118" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE118">
         <v>5</v>
       </c>
-      <c r="IE118">
+      <c r="IF118">
         <v>0.7358867075269341</v>
       </c>
-      <c r="IF118">
+      <c r="IG118">
         <v>0.1293820764152031</v>
       </c>
-      <c r="IG118" t="inlineStr">
+      <c r="IH118" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH118" t="inlineStr">
+      <c r="II118" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -55975,21 +56565,26 @@
       <c r="IC119">
         <v>1</v>
       </c>
-      <c r="ID119">
+      <c r="ID119" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE119">
         <v>6.2</v>
       </c>
-      <c r="IE119">
+      <c r="IF119">
         <v>0.7358867075269341</v>
       </c>
-      <c r="IF119">
+      <c r="IG119">
         <v>0.1293820764152031</v>
       </c>
-      <c r="IG119" t="inlineStr">
+      <c r="IH119" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH119" t="inlineStr">
+      <c r="II119" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -56437,21 +57032,26 @@
       <c r="IC120">
         <v>1</v>
       </c>
-      <c r="ID120">
+      <c r="ID120" t="inlineStr">
+        <is>
+          <t>Reference_1</t>
+        </is>
+      </c>
+      <c r="IE120">
         <v>5.699999999999999</v>
       </c>
-      <c r="IE120">
+      <c r="IF120">
         <v>0.7358867075269341</v>
       </c>
-      <c r="IF120">
+      <c r="IG120">
         <v>0.1293820764152031</v>
       </c>
-      <c r="IG120" t="inlineStr">
+      <c r="IH120" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH120" t="inlineStr">
+      <c r="II120" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
@@ -56890,21 +57490,26 @@
       <c r="IC121">
         <v>1</v>
       </c>
-      <c r="ID121">
+      <c r="ID121" t="inlineStr">
+        <is>
+          <t>Reference_2</t>
+        </is>
+      </c>
+      <c r="IE121">
         <v>5.699999999999999</v>
       </c>
-      <c r="IE121">
+      <c r="IF121">
         <v>0.7358867075269341</v>
       </c>
-      <c r="IF121">
+      <c r="IG121">
         <v>0.1293820764152031</v>
       </c>
-      <c r="IG121" t="inlineStr">
+      <c r="IH121" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="IH121" t="inlineStr">
+      <c r="II121" t="inlineStr">
         <is>
           <t>complete</t>
         </is>

</xml_diff>